<commit_message>
data: GIC segment refresh @ 2026-06-22T08:58Z
</commit_message>
<xml_diff>
--- a/data/raw/gicouncil/segment-annual/FY26-march.xlsx
+++ b/data/raw/gicouncil/segment-annual/FY26-march.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gicouncil-my.sharepoint.com/personal/sskandan_gicouncil_in/Documents/Documents/Year book/25-26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{67E702C2-ED6F-4B82-92D0-94A40279190B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{CBE8E5FD-8548-4BA0-AA48-7DAC20553E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F2E9DD2-ABF4-4565-A869-73C6006C3602}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -426,7 +426,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -473,6 +473,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3111,7 +3112,7 @@
       </c>
       <c r="H5" s="8">
         <f>F5/$F$55</f>
-        <v>7.1591245819751939E-3</v>
+        <v>7.054520699712347E-3</v>
       </c>
       <c r="I5" s="14">
         <f>F5-F6</f>
@@ -3168,7 +3169,7 @@
       </c>
       <c r="H7" s="8">
         <f>F7/$F$55</f>
-        <v>0.12866105067095626</v>
+        <v>0.12678114967997703</v>
       </c>
       <c r="I7" s="14">
         <f>F7-F8</f>
@@ -3225,7 +3226,7 @@
       </c>
       <c r="H9" s="8">
         <f>F9/$F$55</f>
-        <v>4.2721076916564359E-3</v>
+        <v>4.2096867846202098E-3</v>
       </c>
       <c r="I9" s="14">
         <f>F9-F10</f>
@@ -3282,7 +3283,7 @@
       </c>
       <c r="H11" s="8">
         <f>F11/$F$55</f>
-        <v>1.3173601998052746E-2</v>
+        <v>1.2981118979130101E-2</v>
       </c>
       <c r="I11" s="14">
         <f>F11-F12</f>
@@ -3339,7 +3340,7 @@
       </c>
       <c r="H13" s="8">
         <f>F13/$F$55</f>
-        <v>3.7710705668204725E-2</v>
+        <v>3.7159704470977696E-2</v>
       </c>
       <c r="I13" s="14">
         <f>F13-F14</f>
@@ -3396,7 +3397,7 @@
       </c>
       <c r="H15" s="8">
         <f>F15/$F$55</f>
-        <v>0.11776319688439234</v>
+        <v>0.11604252734711312</v>
       </c>
       <c r="I15" s="14">
         <f>F15-F16</f>
@@ -3453,7 +3454,7 @@
       </c>
       <c r="H17" s="8">
         <f>F17/$F$55</f>
-        <v>0.1701731363501672</v>
+        <v>0.16768669118285026</v>
       </c>
       <c r="I17" s="14">
         <f>F17-F18</f>
@@ -3510,7 +3511,7 @@
       </c>
       <c r="H19" s="8">
         <f>F19/$F$55</f>
-        <v>6.290479617322102E-2</v>
+        <v>6.198567738749141E-2</v>
       </c>
       <c r="I19" s="14">
         <f>F19-F20</f>
@@ -3567,7 +3568,7 @@
       </c>
       <c r="H21" s="8">
         <f>F21/$F$55</f>
-        <v>1.4827921940481733E-2</v>
+        <v>1.4611267210828055E-2</v>
       </c>
       <c r="I21" s="14">
         <f>F21-F22</f>
@@ -3678,7 +3679,7 @@
       </c>
       <c r="H25" s="8">
         <f>F25/$F$55</f>
-        <v>8.1158193286204119E-3</v>
+        <v>7.9972369237751358E-3</v>
       </c>
       <c r="I25" s="14">
         <f>F25-F26</f>
@@ -3735,7 +3736,7 @@
       </c>
       <c r="H27" s="8">
         <f>F27/$F$55</f>
-        <v>1.9032299030605764E-2</v>
+        <v>1.8754213023833202E-2</v>
       </c>
       <c r="I27" s="14">
         <f>F27-F28</f>
@@ -3792,7 +3793,7 @@
       </c>
       <c r="H29" s="8">
         <f>F29/$F$55</f>
-        <v>5.1800364051983239E-2</v>
+        <v>5.1043495091201541E-2</v>
       </c>
       <c r="I29" s="14">
         <f>F29-F30</f>
@@ -3903,7 +3904,7 @@
       </c>
       <c r="H33" s="8">
         <f>F33/$F$55</f>
-        <v>1.3168522202937816E-2</v>
+        <v>1.297611340625897E-2</v>
       </c>
       <c r="I33" s="14">
         <f>F33-F34</f>
@@ -3960,7 +3961,7 @@
       </c>
       <c r="H35" s="8">
         <f>F35/$F$55</f>
-        <v>4.9714261524785169E-3</v>
+        <v>4.8987873165457548E-3</v>
       </c>
       <c r="I35" s="14">
         <f>F35-F36</f>
@@ -4017,7 +4018,7 @@
       </c>
       <c r="H37" s="8">
         <f>F37/$F$55</f>
-        <v>2.3434788130212082E-2</v>
+        <v>2.3092376178812414E-2</v>
       </c>
       <c r="I37" s="14">
         <f>F37-F38</f>
@@ -4074,7 +4075,7 @@
       </c>
       <c r="H39" s="8">
         <f>F39/$F$55</f>
-        <v>1.9015366380222664E-3</v>
+        <v>1.8737527780929436E-3</v>
       </c>
       <c r="I39" s="14">
         <f>F39-F40</f>
@@ -4131,7 +4132,7 @@
       </c>
       <c r="H41" s="8">
         <f>F41/$F$55</f>
-        <v>0.14142657579477627</v>
+        <v>0.13936015430512638</v>
       </c>
       <c r="I41" s="14">
         <f>F41-F42</f>
@@ -4188,7 +4189,7 @@
       </c>
       <c r="H43" s="8">
         <f>F43/$F$55</f>
-        <v>0.10421030351775813</v>
+        <v>0.10268765892693867</v>
       </c>
       <c r="I43" s="14">
         <f>F43-F44</f>
@@ -4245,7 +4246,7 @@
       </c>
       <c r="H45" s="8">
         <f>F45/$F$55</f>
-        <v>2.7945646192270242E-2</v>
+        <v>2.7537324888375726E-2</v>
       </c>
       <c r="I45" s="14">
         <f>F45-F46</f>
@@ -4302,7 +4303,7 @@
       </c>
       <c r="H47" s="8">
         <f>F47/$F$55</f>
-        <v>4.8061634847394494E-2</v>
+        <v>4.7359393458049973E-2</v>
       </c>
       <c r="I47" s="14">
         <f>F47-F48</f>
@@ -4359,7 +4360,7 @@
       </c>
       <c r="H49" s="8">
         <f>F49/$F$55</f>
-        <v>4.8308851542987769E-3</v>
+        <v>4.7602998004444954E-3</v>
       </c>
       <c r="I49" s="14">
         <f>F49-F50</f>
@@ -4416,7 +4417,7 @@
       </c>
       <c r="H51" s="8">
         <f>F51/$F$55</f>
-        <v>3.2172035727892307E-5</v>
+        <v>3.1701961517155772E-5</v>
       </c>
       <c r="I51" s="14">
         <f>F51-F52</f>
@@ -4473,7 +4474,7 @@
       </c>
       <c r="H53" s="8">
         <f>F53/$F$55</f>
-        <v>9.2503069042881945E-3</v>
+        <v>9.1151481983274725E-3</v>
       </c>
       <c r="I53" s="14">
         <f>F53-F54</f>
@@ -4509,23 +4510,28 @@
         <v>36</v>
       </c>
       <c r="B55" s="5">
-        <v>1009.34</v>
+        <f t="shared" ref="B55:F56" si="1">SUM(B5+B7+B9+B11+B13+B15+B17+B19+B21+B23+B25+B27+B29+B31+B33+B35+B37+B39+B41+B43+B45+B47+B49+B51+B53)</f>
+        <v>1032.0700000000002</v>
       </c>
       <c r="C55" s="5">
-        <v>166.93</v>
+        <f t="shared" si="1"/>
+        <v>170.5</v>
       </c>
       <c r="D55" s="5">
-        <v>235.8</v>
+        <f t="shared" si="1"/>
+        <v>236.66</v>
       </c>
       <c r="E55" s="5">
-        <v>4493.68</v>
+        <f t="shared" si="1"/>
+        <v>4554.0900000000011</v>
       </c>
       <c r="F55" s="5">
-        <v>5905.75</v>
+        <f t="shared" si="1"/>
+        <v>5993.32</v>
       </c>
       <c r="G55" s="11">
         <f>F55/F56-1</f>
-        <v>9.7461942140159907E-2</v>
+        <v>9.5969468831546445E-2</v>
       </c>
       <c r="H55" s="12">
         <f>F55/$F$55</f>
@@ -4533,7 +4539,7 @@
       </c>
       <c r="I55" s="7">
         <f>F55-F56</f>
-        <v>524.47000000000025</v>
+        <v>524.8100000000004</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
@@ -4541,19 +4547,24 @@
         <v>37</v>
       </c>
       <c r="B56" s="4">
-        <v>905.88</v>
+        <f t="shared" si="1"/>
+        <v>935.51</v>
       </c>
       <c r="C56" s="4">
-        <v>112.74</v>
+        <f t="shared" si="1"/>
+        <v>114.19999999999996</v>
       </c>
       <c r="D56" s="4">
-        <v>236.88</v>
+        <f t="shared" si="1"/>
+        <v>237.62999999999994</v>
       </c>
       <c r="E56" s="4">
-        <v>4125.78</v>
+        <f t="shared" si="1"/>
+        <v>4181.170000000001</v>
       </c>
       <c r="F56" s="4">
-        <v>5381.28</v>
+        <f t="shared" si="1"/>
+        <v>5468.5099999999993</v>
       </c>
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
@@ -4565,23 +4576,23 @@
       </c>
       <c r="B57" s="9">
         <f>B55/B56-1</f>
-        <v>0.11420938755685084</v>
+        <v>0.10321642740323478</v>
       </c>
       <c r="C57" s="9">
-        <f t="shared" ref="C57:F57" si="1">C55/C56-1</f>
-        <v>0.4806634734788009</v>
+        <f t="shared" ref="C57:F57" si="2">C55/C56-1</f>
+        <v>0.49299474605954519</v>
       </c>
       <c r="D57" s="9">
-        <f t="shared" si="1"/>
-        <v>-4.5592705167172287E-3</v>
+        <f t="shared" si="2"/>
+        <v>-4.0819761814583355E-3</v>
       </c>
       <c r="E57" s="9">
-        <f t="shared" si="1"/>
-        <v>8.9171017359142013E-2</v>
+        <f t="shared" si="2"/>
+        <v>8.9190346242798091E-2</v>
       </c>
       <c r="F57" s="9">
-        <f t="shared" si="1"/>
-        <v>9.7461942140159907E-2</v>
+        <f t="shared" si="2"/>
+        <v>9.5969468831546445E-2</v>
       </c>
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
@@ -4593,22 +4604,22 @@
       </c>
       <c r="B58" s="8">
         <f>B55/$F$55</f>
-        <v>0.17090801337679382</v>
+        <v>0.17220338643689978</v>
       </c>
       <c r="C58" s="8">
-        <f t="shared" ref="C58:F58" si="2">C55/$F$55</f>
-        <v>2.8265673284510861E-2</v>
+        <f t="shared" ref="C58:F58" si="3">C55/$F$55</f>
+        <v>2.8448339150921362E-2</v>
       </c>
       <c r="D58" s="8">
-        <f t="shared" si="2"/>
-        <v>3.9927189603352668E-2</v>
+        <f t="shared" si="3"/>
+        <v>3.9487295856053074E-2</v>
       </c>
       <c r="E58" s="8">
-        <f t="shared" si="2"/>
-        <v>0.76089912373534274</v>
+        <f t="shared" si="3"/>
+        <v>0.759860978556126</v>
       </c>
       <c r="F58" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G58" s="1"/>
@@ -4621,22 +4632,22 @@
       </c>
       <c r="B59" s="8">
         <f>B56/$F$56</f>
-        <v>0.16833913121041835</v>
+        <v>0.17107219333968487</v>
       </c>
       <c r="C59" s="8">
-        <f t="shared" ref="C59:F59" si="3">C56/$F$56</f>
-        <v>2.0950405851395952E-2</v>
+        <f t="shared" ref="C59:F59" si="4">C56/$F$56</f>
+        <v>2.0883202188530327E-2</v>
       </c>
       <c r="D59" s="8">
-        <f t="shared" si="3"/>
-        <v>4.4019266791544019E-2</v>
+        <f t="shared" si="4"/>
+        <v>4.3454249877937494E-2</v>
       </c>
       <c r="E59" s="8">
-        <f t="shared" si="3"/>
-        <v>0.76669119614664172</v>
+        <f t="shared" si="4"/>
+        <v>0.76459035459384761</v>
       </c>
       <c r="F59" s="8">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="G59" s="1"/>
@@ -4735,7 +4746,7 @@
       </c>
       <c r="G4" s="8">
         <f>E4/$E$65</f>
-        <v>3.8266741313398266E-3</v>
+        <v>3.4934702953242935E-3</v>
       </c>
       <c r="H4" s="14">
         <f>E4-E5</f>
@@ -4786,7 +4797,7 @@
       </c>
       <c r="G6" s="8">
         <f>E6/$E$65</f>
-        <v>9.273312695707539E-2</v>
+        <v>8.4658482352572742E-2</v>
       </c>
       <c r="H6" s="14">
         <f>E6-E7</f>
@@ -4837,7 +4848,7 @@
       </c>
       <c r="G8" s="8">
         <f>E8/$E$65</f>
-        <v>1.604767511107818E-3</v>
+        <v>1.4650339795183366E-3</v>
       </c>
       <c r="H8" s="14">
         <f>E8-E9</f>
@@ -4888,7 +4899,7 @@
       </c>
       <c r="G10" s="8">
         <f>E10/$E$65</f>
-        <v>2.0490116168976048E-2</v>
+        <v>1.8705959725658451E-2</v>
       </c>
       <c r="H10" s="14">
         <f>E10-E11</f>
@@ -4939,7 +4950,7 @@
       </c>
       <c r="G12" s="8">
         <f>E12/$E$65</f>
-        <v>7.0255747386678306E-3</v>
+        <v>6.4138298205505635E-3</v>
       </c>
       <c r="H12" s="14">
         <f>E12-E13</f>
@@ -4990,7 +5001,7 @@
       </c>
       <c r="G14" s="8">
         <f>E14/$E$65</f>
-        <v>6.5377638364029059E-2</v>
+        <v>5.9684945664088204E-2</v>
       </c>
       <c r="H14" s="14">
         <f>E14-E15</f>
@@ -5041,7 +5052,7 @@
       </c>
       <c r="G16" s="8">
         <f>E16/$E$65</f>
-        <v>4.8933059445693129E-2</v>
+        <v>4.4672262065077822E-2</v>
       </c>
       <c r="H16" s="14">
         <f>E16-E17</f>
@@ -5092,7 +5103,7 @@
       </c>
       <c r="G18" s="8">
         <f>E18/$E$65</f>
-        <v>4.8543359596907656E-2</v>
+        <v>4.4316494942219169E-2</v>
       </c>
       <c r="H18" s="14">
         <f>E18-E19</f>
@@ -5143,7 +5154,7 @@
       </c>
       <c r="G20" s="8">
         <f>E20/$E$65</f>
-        <v>9.5379037990246524E-2</v>
+        <v>8.7074003319658005E-2</v>
       </c>
       <c r="H20" s="14">
         <f>E20-E21</f>
@@ -5194,7 +5205,7 @@
       </c>
       <c r="G22" s="8">
         <f>E22/$E$65</f>
-        <v>3.4488779663156624E-2</v>
+        <v>3.1485703548275977E-2</v>
       </c>
       <c r="H22" s="14">
         <f>E22-E23</f>
@@ -5245,7 +5256,7 @@
       </c>
       <c r="G24" s="8">
         <f>E24/$E$65</f>
-        <v>2.9038813556066011E-3</v>
+        <v>2.6510287808086189E-3</v>
       </c>
       <c r="H24" s="14">
         <f>E24-E25</f>
@@ -5296,7 +5307,7 @@
       </c>
       <c r="G26" s="8">
         <f>E26/$E$65</f>
-        <v>1.4596592047378719E-3</v>
+        <v>1.3325608342989572E-3</v>
       </c>
       <c r="H26" s="14">
         <f>E26-E27</f>
@@ -5347,7 +5358,7 @@
       </c>
       <c r="G28" s="8">
         <f>E28/$E$65</f>
-        <v>1.5746137992167581E-2</v>
+        <v>1.4375058720365791E-2</v>
       </c>
       <c r="H28" s="14">
         <f>E28-E29</f>
@@ -5446,7 +5457,7 @@
       </c>
       <c r="G32" s="8">
         <f>E32/$E$65</f>
-        <v>4.9604399766180099E-4</v>
+        <v>4.5285146096270089E-4</v>
       </c>
       <c r="H32" s="14">
         <f>E32-E33</f>
@@ -5497,7 +5508,7 @@
       </c>
       <c r="G34" s="8">
         <f>E34/$E$65</f>
-        <v>9.5126556398075659E-4</v>
+        <v>8.6843506310481985E-4</v>
       </c>
       <c r="H34" s="14">
         <f>E34-E35</f>
@@ -5548,7 +5559,7 @@
       </c>
       <c r="G36" s="8">
         <f>E36/$E$65</f>
-        <v>7.2688970122096797E-2</v>
+        <v>6.635965049638283E-2</v>
       </c>
       <c r="H36" s="14">
         <f>E36-E37</f>
@@ -5599,7 +5610,7 @@
       </c>
       <c r="G38" s="8">
         <f>E38/$E$65</f>
-        <v>1.6569104486213681E-3</v>
+        <v>1.5126366227177352E-3</v>
       </c>
       <c r="H38" s="14">
         <f>E38-E39</f>
@@ -5650,7 +5661,7 @@
       </c>
       <c r="G40" s="8">
         <f>E40/$E$65</f>
-        <v>4.7573569568283923E-2</v>
+        <v>4.343114841376719E-2</v>
       </c>
       <c r="H40" s="14">
         <f>E40-E41</f>
@@ -5701,7 +5712,7 @@
       </c>
       <c r="G42" s="8">
         <f>E42/$E$65</f>
-        <v>6.1135192915146977E-2</v>
+        <v>5.5811906924305543E-2</v>
       </c>
       <c r="H42" s="14">
         <f>E42-E43</f>
@@ -5752,7 +5763,7 @@
       </c>
       <c r="G44" s="8">
         <f>E44/$E$65</f>
-        <v>2.6537667783623275E-2</v>
+        <v>2.4226926810936081E-2</v>
       </c>
       <c r="H44" s="14">
         <f>E44-E45</f>
@@ -5803,7 +5814,7 @@
       </c>
       <c r="G46" s="8">
         <f>E46/$E$65</f>
-        <v>1.8942294234363295E-2</v>
+        <v>1.7292912843318409E-2</v>
       </c>
       <c r="H46" s="14">
         <f>E46-E47</f>
@@ -5854,7 +5865,7 @@
       </c>
       <c r="G48" s="8">
         <f>E48/$E$65</f>
-        <v>1.9641078206173175E-2</v>
+        <v>1.7930850897247191E-2</v>
       </c>
       <c r="H48" s="14">
         <f>E48-E49</f>
@@ -5905,7 +5916,7 @@
       </c>
       <c r="G50" s="8">
         <f>E50/$E$65</f>
-        <v>2.149523989867804E-3</v>
+        <v>1.9623563308383703E-3</v>
       </c>
       <c r="H50" s="14">
         <f>E50-E51</f>
@@ -5956,7 +5967,7 @@
       </c>
       <c r="G52" s="8">
         <f>E52/$E$65</f>
-        <v>2.3567235573558592E-3</v>
+        <v>2.1515142024991392E-3</v>
       </c>
       <c r="H52" s="14">
         <f>E52-E53</f>
@@ -5989,25 +6000,28 @@
         <v>36</v>
       </c>
       <c r="B54" s="5">
-        <v>9025.19</v>
+        <f t="shared" ref="B54:E55" si="1">SUM(B4+B6+B8+B10+B12+B14+B16+B18+B20+B22+B24+B26+B28+B30+B32+B34+B36+B38+B40+B42+B44+B46+B48+B50+B52)</f>
+        <v>11712.33</v>
       </c>
       <c r="C54" s="5">
+        <f t="shared" si="1"/>
         <v>897.95</v>
       </c>
       <c r="D54" s="5">
-        <v>7487.43</v>
+        <f t="shared" si="1"/>
+        <v>7580.6500000000005</v>
       </c>
       <c r="E54" s="5">
-        <f t="shared" si="0"/>
-        <v>17410.57</v>
+        <f t="shared" si="1"/>
+        <v>20190.929999999997</v>
       </c>
       <c r="F54" s="11">
         <f>E54/E55-1</f>
-        <v>-0.26590397950501365</v>
+        <v>-0.26999978307084926</v>
       </c>
       <c r="G54" s="12">
         <f>E54/$E$65</f>
-        <v>0.59726201551664049</v>
+        <v>0.6323300241144969</v>
       </c>
       <c r="H54" s="3">
         <v>-6306.45</v>
@@ -6018,17 +6032,20 @@
         <v>37</v>
       </c>
       <c r="B55" s="4">
-        <v>16574.849999999999</v>
+        <f t="shared" si="1"/>
+        <v>20430.79</v>
       </c>
       <c r="C55" s="4">
+        <f t="shared" si="1"/>
         <v>768.85</v>
       </c>
       <c r="D55" s="4">
-        <v>6373.32</v>
+        <f t="shared" si="1"/>
+        <v>6459.16</v>
       </c>
       <c r="E55" s="4">
-        <f t="shared" si="0"/>
-        <v>23717.019999999997</v>
+        <f t="shared" si="1"/>
+        <v>27658.800000000003</v>
       </c>
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
@@ -6040,19 +6057,19 @@
       </c>
       <c r="B56" s="11">
         <f>B54/B55-1</f>
-        <v>-0.45548888828556511</v>
+        <v>-0.4267314186088742</v>
       </c>
       <c r="C56" s="11">
-        <f t="shared" ref="C56:E56" si="1">C54/C55-1</f>
+        <f t="shared" ref="C56:E56" si="2">C54/C55-1</f>
         <v>0.16791311699291156</v>
       </c>
       <c r="D56" s="11">
-        <f t="shared" si="1"/>
-        <v>0.17480842010129738</v>
+        <f t="shared" si="2"/>
+        <v>0.1736278401525897</v>
       </c>
       <c r="E56" s="11">
-        <f t="shared" si="1"/>
-        <v>-0.26590397950501365</v>
+        <f t="shared" si="2"/>
+        <v>-0.26999978307084926</v>
       </c>
       <c r="F56" s="1"/>
       <c r="G56" s="1"/>
@@ -6084,7 +6101,7 @@
         <v>88.69</v>
       </c>
       <c r="E58" s="5">
-        <f t="shared" ref="E58:E61" si="2">SUM(B58:D58)</f>
+        <f t="shared" ref="E58:E61" si="3">SUM(B58:D58)</f>
         <v>10279.99</v>
       </c>
       <c r="F58" s="13">
@@ -6093,7 +6110,7 @@
       </c>
       <c r="G58" s="6">
         <f>E58/$E$65</f>
-        <v>0.35265057645389603</v>
+        <v>0.32194387898907023</v>
       </c>
       <c r="H58" s="1">
         <v>541.83000000000004</v>
@@ -6113,7 +6130,7 @@
         <v>77.97</v>
       </c>
       <c r="E59" s="15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9738.16</v>
       </c>
       <c r="F59" s="1"/>
@@ -6134,7 +6151,7 @@
         <v>0</v>
       </c>
       <c r="E60" s="5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1460.08</v>
       </c>
       <c r="F60" s="13">
@@ -6143,7 +6160,7 @@
       </c>
       <c r="G60" s="6">
         <f>E60/$E$65</f>
-        <v>5.0087408029463501E-2</v>
+        <v>4.5726096896432936E-2</v>
       </c>
       <c r="H60" s="1">
         <v>93.53</v>
@@ -6163,7 +6180,7 @@
         <v>0</v>
       </c>
       <c r="E61" s="15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1366.55</v>
       </c>
       <c r="F61" s="1"/>
@@ -6175,12 +6192,15 @@
         <v>62</v>
       </c>
       <c r="B62" s="5">
+        <f>B58+B60</f>
         <v>10191.299999999999</v>
       </c>
       <c r="C62" s="5">
+        <f t="shared" ref="C62:D62" si="4">C58+C60</f>
         <v>1460.08</v>
       </c>
       <c r="D62" s="5">
+        <f t="shared" si="4"/>
         <v>88.69</v>
       </c>
       <c r="E62" s="5">
@@ -6192,7 +6212,7 @@
       </c>
       <c r="G62" s="12">
         <f>E62/$E$65</f>
-        <v>0.40273798448335951</v>
+        <v>0.36766997588550315</v>
       </c>
       <c r="H62" s="3">
         <v>635.36</v>
@@ -6203,15 +6223,19 @@
         <v>37</v>
       </c>
       <c r="B63" s="4">
+        <f>B59+B61</f>
         <v>9660.19</v>
       </c>
       <c r="C63" s="4">
+        <f t="shared" ref="C63:E63" si="5">C59+C61</f>
         <v>1366.55</v>
       </c>
       <c r="D63" s="4">
+        <f t="shared" si="5"/>
         <v>77.97</v>
       </c>
       <c r="E63" s="4">
+        <f t="shared" si="5"/>
         <v>11104.71</v>
       </c>
       <c r="F63" s="1"/>
@@ -6227,15 +6251,15 @@
         <v>5.4979249890529935E-2</v>
       </c>
       <c r="C64" s="11">
-        <f t="shared" ref="C64:E64" si="3">C62/C63-1</f>
+        <f t="shared" ref="C64:E64" si="6">C62/C63-1</f>
         <v>6.8442428012147394E-2</v>
       </c>
       <c r="D64" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>0.13748877773502621</v>
       </c>
       <c r="E64" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>5.7215361769915596E-2</v>
       </c>
       <c r="F64" s="1"/>
@@ -6248,23 +6272,23 @@
       </c>
       <c r="B65" s="7">
         <f>B62+B54</f>
-        <v>19216.489999999998</v>
+        <v>21903.629999999997</v>
       </c>
       <c r="C65" s="7">
-        <f t="shared" ref="C65:E65" si="4">C62+C54</f>
+        <f t="shared" ref="C65:E65" si="7">C62+C54</f>
         <v>2358.0299999999997</v>
       </c>
       <c r="D65" s="7">
-        <f t="shared" si="4"/>
-        <v>7576.12</v>
+        <f t="shared" si="7"/>
+        <v>7669.34</v>
       </c>
       <c r="E65" s="7">
-        <f t="shared" si="4"/>
-        <v>29150.639999999999</v>
+        <f t="shared" si="7"/>
+        <v>31930.999999999996</v>
       </c>
       <c r="F65" s="11">
         <f>E65/E66-1</f>
-        <v>-0.16286066200616678</v>
+        <v>-0.17626138603031571</v>
       </c>
       <c r="G65" s="12">
         <f>E65/$E$65</f>
@@ -6280,19 +6304,19 @@
       </c>
       <c r="B66" s="14">
         <f>B63+B55</f>
-        <v>26235.040000000001</v>
+        <v>30090.980000000003</v>
       </c>
       <c r="C66" s="14">
-        <f t="shared" ref="C66:E66" si="5">C63+C55</f>
+        <f t="shared" ref="C66:E66" si="8">C63+C55</f>
         <v>2135.4</v>
       </c>
       <c r="D66" s="14">
-        <f t="shared" si="5"/>
-        <v>6451.29</v>
+        <f t="shared" si="8"/>
+        <v>6537.13</v>
       </c>
       <c r="E66" s="14">
-        <f t="shared" si="5"/>
-        <v>34821.729999999996</v>
+        <f t="shared" si="8"/>
+        <v>38763.51</v>
       </c>
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
@@ -10566,7 +10590,7 @@
         <v>0.05</v>
       </c>
       <c r="O72" s="5">
-        <f t="shared" ref="O58:O73" si="7">B72+C72+F72+G72+J72+L72+M72+N72</f>
+        <f t="shared" ref="O72:O73" si="7">B72+C72+F72+G72+J72+L72+M72+N72</f>
         <v>45865.94</v>
       </c>
       <c r="P72" s="11">
@@ -11357,9 +11381,9 @@
         <f t="shared" si="12"/>
         <v>9.4998201251995248E-2</v>
       </c>
-      <c r="O86" s="9">
-        <f t="shared" ref="O86:O87" si="13">B86+C86+F86+G86+J86+L86+M86+N86</f>
-        <v>0.99675930823828962</v>
+      <c r="O86" s="26">
+        <f>B86+C86+F86+G86+J86+K86+L86+M86+N86</f>
+        <v>1</v>
       </c>
       <c r="P86" s="16"/>
       <c r="Q86" s="1"/>
@@ -11374,56 +11398,56 @@
         <v>7.8870427027905296E-2</v>
       </c>
       <c r="C87" s="8">
-        <f t="shared" ref="C87:N87" si="14">C84/$O$84</f>
+        <f t="shared" ref="C87:N87" si="13">C84/$O$84</f>
         <v>1.7889643295020883E-2</v>
       </c>
       <c r="D87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1.2807096025169802E-2</v>
       </c>
       <c r="E87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>5.0825472698510805E-3</v>
       </c>
       <c r="F87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1.9551799093995396E-2</v>
       </c>
       <c r="G87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0.32208687434199018</v>
       </c>
       <c r="H87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0.13116232041213968</v>
       </c>
       <c r="I87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0.19092455392985042</v>
       </c>
       <c r="J87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0.38632699549623967</v>
       </c>
       <c r="K87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>3.5683791777233538E-3</v>
       </c>
       <c r="L87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1.7774483961535671E-2</v>
       </c>
       <c r="M87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>2.7936490683941446E-2</v>
       </c>
       <c r="N87" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0.12599490692164797</v>
       </c>
-      <c r="O87" s="9">
-        <f t="shared" si="13"/>
-        <v>0.99643162082227654</v>
+      <c r="O87" s="26">
+        <f>B87+C87+F87+G87+J87+K87+L87+M87+N87</f>
+        <v>0.99999999999999989</v>
       </c>
       <c r="P87" s="1"/>
       <c r="Q87" s="1"/>

</xml_diff>